<commit_message>
Changed relevancy condition for breastfedding questions
</commit_message>
<xml_diff>
--- a/forms/app/infant_child.xlsx
+++ b/forms/app/infant_child.xlsx
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="Z_781EBA2C_D8B1_4B7C_8F0C_A942CACA9398_.wvu.FilterData" localSheetId="0" hidden="1">survey!$A$389:$Z$420</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
   <customWorkbookViews>
     <customWorkbookView name="Filter 1" guid="{781EBA2C-D8B1-4B7C-8F0C-A942CACA9398}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
   </customWorkbookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2617" uniqueCount="1652">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2617" uniqueCount="1653">
   <si>
     <t>type</t>
   </si>
@@ -5425,6 +5425,10 @@
   </si>
   <si>
     <t>data</t>
+  </si>
+  <si>
+    <t>&lt;span style="color:#f58a1f;font-weight: bold"&gt;If possible, ask the mother to breastfeed and observe. If not possible, ask questions below rather than observing.WASH your hands. OBSERVE the mother breastfeeding. Try to UNDERSTAND the situation.Do you notice any problems with breastfeeding? Provide guidance based on what you observe. Try to solve any problems you identify or the mother describes.&lt;/span&gt;
+&lt;span style="color:#f58a1f;display:block;padding-left:1em"&gt;Je umegundua kuna tatizo lolote kwenye kunyonyesha? Toa muongozo kwa kile ulichokiona. Jaribu kutatua tatizo lolote uliloliona au alilolisema mama.&lt;/span&gt;</t>
   </si>
 </sst>
 </file>
@@ -5514,7 +5518,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -5567,6 +5571,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11243,8 +11250,8 @@
       <c r="B195" s="1" t="s">
         <v>502</v>
       </c>
-      <c r="C195" s="18" t="s">
-        <v>503</v>
+      <c r="C195" s="48" t="s">
+        <v>1652</v>
       </c>
       <c r="D195" s="18" t="s">
         <v>503</v>
@@ -12314,7 +12321,7 @@
         <v>169</v>
       </c>
       <c r="F232" s="4" t="s">
-        <v>599</v>
+        <v>606</v>
       </c>
       <c r="G232" s="6"/>
       <c r="H232" s="6"/>
@@ -20037,6 +20044,19 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="21">
+    <mergeCell ref="K275:L275"/>
+    <mergeCell ref="F276:G276"/>
+    <mergeCell ref="K279:L279"/>
+    <mergeCell ref="K282:L282"/>
+    <mergeCell ref="K285:L285"/>
+    <mergeCell ref="K288:L288"/>
+    <mergeCell ref="K291:L291"/>
+    <mergeCell ref="F313:H313"/>
+    <mergeCell ref="F314:H314"/>
+    <mergeCell ref="F328:I328"/>
+    <mergeCell ref="K315:L315"/>
+    <mergeCell ref="K318:L318"/>
+    <mergeCell ref="K321:L321"/>
     <mergeCell ref="L331:O331"/>
     <mergeCell ref="K294:L294"/>
     <mergeCell ref="K297:L297"/>
@@ -20045,19 +20065,6 @@
     <mergeCell ref="K306:L306"/>
     <mergeCell ref="K309:L309"/>
     <mergeCell ref="K312:L312"/>
-    <mergeCell ref="K288:L288"/>
-    <mergeCell ref="K291:L291"/>
-    <mergeCell ref="F313:H313"/>
-    <mergeCell ref="F314:H314"/>
-    <mergeCell ref="F328:I328"/>
-    <mergeCell ref="K315:L315"/>
-    <mergeCell ref="K318:L318"/>
-    <mergeCell ref="K321:L321"/>
-    <mergeCell ref="K275:L275"/>
-    <mergeCell ref="F276:G276"/>
-    <mergeCell ref="K279:L279"/>
-    <mergeCell ref="K282:L282"/>
-    <mergeCell ref="K285:L285"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Re-arranged relevancy condition in breastfeeding section
</commit_message>
<xml_diff>
--- a/forms/app/infant_child.xlsx
+++ b/forms/app/infant_child.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2568" uniqueCount="1633">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2569" uniqueCount="1633">
   <si>
     <t>type</t>
   </si>
@@ -5230,9 +5230,6 @@
     <t xml:space="preserve">Essential New Born Care: Breastfeeding </t>
   </si>
   <si>
-    <t>not(selected(${child_consent_today},"no")) and ${age_days} &lt;= (${month} * 24) and ${refer_neonatal_danger_sign_flag}=0 and ${refer_child_danger_sign_flag}=0</t>
-  </si>
-  <si>
     <t>small_baby_intro</t>
   </si>
   <si>
@@ -5274,9 +5271,6 @@
   </si>
   <si>
     <t xml:space="preserve">Zungumza na mama kuhusu tatizo na msaidie kulitatua. </t>
-  </si>
-  <si>
-    <t>selected(${baby_breastfeed_well},"no") and  ${small_baby_ever}=1 and  ${age_days} &lt;= (${month} * 6)</t>
   </si>
   <si>
     <t>not_breastfeeding_well</t>
@@ -5336,9 +5330,6 @@
     <t>${n_child_visits} = 0 and ${age_days} &lt; (${month} * 6)</t>
   </si>
   <si>
-    <t>selected(${baby_breastfeed_well},"no") and  (${small_baby_ever}=0 or ${small_baby_ever}=1 and  ${age_days} &lt;= (${month} * 6))</t>
-  </si>
-  <si>
     <t>selected(${baby_times_breastfed_daily},"five_more_times_day")</t>
   </si>
   <si>
@@ -5361,6 +5352,15 @@
   </si>
   <si>
     <t>selected(${currently_breastfeeding},"yes") and ${age_days} &lt; (${month} * 6) and ${random_value} &gt; 5</t>
+  </si>
+  <si>
+    <t>selected(${baby_breastfeed_well},"no") and  ${small_baby_ever}=1 and  ${age_days} &lt; (${month} * 6)</t>
+  </si>
+  <si>
+    <t>selected(${baby_breastfeed_well},"no") and  (${small_baby_ever}=0 or ${small_baby_ever}=1 and  ${age_days} &lt; (${month} * 6))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${age_days} &lt;= (${month} * 24) </t>
   </si>
 </sst>
 </file>
@@ -5371,7 +5371,7 @@
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -5407,6 +5407,11 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -5440,7 +5445,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -5476,6 +5481,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11028,8 +11035,8 @@
       <c r="D188" s="2" t="s">
         <v>479</v>
       </c>
-      <c r="F188" s="19" t="s">
-        <v>1592</v>
+      <c r="F188" s="23" t="s">
+        <v>401</v>
       </c>
     </row>
     <row r="189" spans="1:17" ht="78">
@@ -11037,16 +11044,16 @@
         <v>139</v>
       </c>
       <c r="B189" s="1" t="s">
+        <v>1592</v>
+      </c>
+      <c r="C189" s="18" t="s">
+        <v>1594</v>
+      </c>
+      <c r="D189" s="10" t="s">
         <v>1593</v>
       </c>
-      <c r="C189" s="18" t="s">
-        <v>1595</v>
-      </c>
-      <c r="D189" s="10" t="s">
-        <v>1594</v>
-      </c>
       <c r="F189" s="19" t="s">
-        <v>1601</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="190" spans="1:17" ht="65">
@@ -11064,7 +11071,7 @@
       </c>
       <c r="E190" s="1"/>
       <c r="F190" s="2" t="s">
-        <v>1622</v>
+        <v>1620</v>
       </c>
       <c r="G190" s="1"/>
       <c r="H190" s="1"/>
@@ -11095,7 +11102,7 @@
         <v>171</v>
       </c>
       <c r="F191" s="1" t="s">
-        <v>1623</v>
+        <v>1621</v>
       </c>
       <c r="G191" s="1"/>
       <c r="H191" s="1"/>
@@ -11156,7 +11163,9 @@
       <c r="E193" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="F193" s="1"/>
+      <c r="F193" s="24" t="s">
+        <v>1632</v>
+      </c>
       <c r="G193" s="1"/>
       <c r="H193" s="1"/>
       <c r="I193" s="1"/>
@@ -11206,10 +11215,10 @@
         <v>498</v>
       </c>
       <c r="C195" s="10" t="s">
+        <v>1596</v>
+      </c>
+      <c r="D195" s="10" t="s">
         <v>1597</v>
-      </c>
-      <c r="D195" s="10" t="s">
-        <v>1598</v>
       </c>
       <c r="E195" s="1"/>
       <c r="F195" s="2" t="s">
@@ -11235,7 +11244,7 @@
         <v>499</v>
       </c>
       <c r="C196" s="10" t="s">
-        <v>1596</v>
+        <v>1595</v>
       </c>
       <c r="D196" s="10" t="s">
         <v>500</v>
@@ -11261,7 +11270,7 @@
         <v>167</v>
       </c>
       <c r="B197" s="1" t="s">
-        <v>1599</v>
+        <v>1598</v>
       </c>
       <c r="C197" s="3" t="s">
         <v>566</v>
@@ -11290,16 +11299,16 @@
         <v>139</v>
       </c>
       <c r="B198" s="1" t="s">
-        <v>1606</v>
+        <v>1604</v>
       </c>
       <c r="C198" s="20" t="s">
-        <v>1600</v>
+        <v>1599</v>
       </c>
       <c r="D198" s="20" t="s">
-        <v>1607</v>
+        <v>1605</v>
       </c>
       <c r="F198" s="19" t="s">
-        <v>1624</v>
+        <v>1631</v>
       </c>
     </row>
     <row r="199" spans="1:17">
@@ -11307,16 +11316,16 @@
         <v>139</v>
       </c>
       <c r="B199" s="1" t="s">
+        <v>1601</v>
+      </c>
+      <c r="C199" s="18" t="s">
         <v>1602</v>
       </c>
-      <c r="C199" s="18" t="s">
+      <c r="D199" s="18" t="s">
         <v>1603</v>
       </c>
-      <c r="D199" s="18" t="s">
-        <v>1604</v>
-      </c>
       <c r="F199" s="19" t="s">
-        <v>1605</v>
+        <v>1630</v>
       </c>
     </row>
     <row r="200" spans="1:17">
@@ -11324,13 +11333,13 @@
         <v>62</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>1608</v>
+        <v>1606</v>
       </c>
       <c r="C200" s="18"/>
       <c r="D200" s="18"/>
       <c r="F200" s="19"/>
       <c r="L200" t="s">
-        <v>1630</v>
+        <v>1627</v>
       </c>
     </row>
     <row r="201" spans="1:17">
@@ -11338,7 +11347,7 @@
         <v>167</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>1627</v>
+        <v>1624</v>
       </c>
       <c r="C201" s="2" t="s">
         <v>501</v>
@@ -11350,7 +11359,7 @@
         <v>171</v>
       </c>
       <c r="F201" s="2" t="s">
-        <v>1631</v>
+        <v>1628</v>
       </c>
       <c r="G201" s="2"/>
       <c r="H201" s="1"/>
@@ -11366,19 +11375,19 @@
     </row>
     <row r="202" spans="1:17">
       <c r="A202" s="1" t="s">
-        <v>1612</v>
+        <v>1610</v>
       </c>
       <c r="B202" s="1" t="s">
+        <v>1607</v>
+      </c>
+      <c r="C202" t="s">
+        <v>1608</v>
+      </c>
+      <c r="D202" t="s">
         <v>1609</v>
       </c>
-      <c r="C202" t="s">
-        <v>1610</v>
-      </c>
-      <c r="D202" t="s">
-        <v>1611</v>
-      </c>
       <c r="F202" s="2" t="s">
-        <v>1632</v>
+        <v>1629</v>
       </c>
     </row>
     <row r="203" spans="1:17">
@@ -11386,16 +11395,16 @@
         <v>139</v>
       </c>
       <c r="B203" s="1" t="s">
+        <v>1611</v>
+      </c>
+      <c r="C203" t="s">
+        <v>1612</v>
+      </c>
+      <c r="D203" t="s">
         <v>1613</v>
       </c>
-      <c r="C203" t="s">
+      <c r="F203" s="19" t="s">
         <v>1614</v>
-      </c>
-      <c r="D203" t="s">
-        <v>1615</v>
-      </c>
-      <c r="F203" s="19" t="s">
-        <v>1616</v>
       </c>
     </row>
     <row r="204" spans="1:17">
@@ -11403,7 +11412,7 @@
         <v>561</v>
       </c>
       <c r="B204" s="1" t="s">
-        <v>1618</v>
+        <v>1616</v>
       </c>
       <c r="C204" s="3" t="s">
         <v>562</v>
@@ -11415,7 +11424,7 @@
         <v>171</v>
       </c>
       <c r="F204" s="2" t="s">
-        <v>1617</v>
+        <v>1615</v>
       </c>
       <c r="G204" s="2"/>
       <c r="H204" s="2"/>
@@ -11434,7 +11443,7 @@
         <v>139</v>
       </c>
       <c r="B205" s="1" t="s">
-        <v>1619</v>
+        <v>1617</v>
       </c>
       <c r="C205" s="10" t="s">
         <v>564</v>
@@ -11444,7 +11453,7 @@
       </c>
       <c r="E205" s="1"/>
       <c r="F205" s="2" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="G205" s="2"/>
       <c r="H205" s="2"/>
@@ -11463,13 +11472,13 @@
         <v>139</v>
       </c>
       <c r="B206" s="1" t="s">
-        <v>1620</v>
+        <v>1618</v>
       </c>
       <c r="C206" t="s">
-        <v>1621</v>
+        <v>1619</v>
       </c>
       <c r="F206" s="2" t="s">
-        <v>1626</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="207" spans="1:17">
@@ -12777,7 +12786,7 @@
         <v>139</v>
       </c>
       <c r="B254" s="1" t="s">
-        <v>1628</v>
+        <v>1625</v>
       </c>
       <c r="C254" s="10"/>
       <c r="D254" s="10"/>
@@ -12797,10 +12806,10 @@
       <c r="P254" s="1"/>
       <c r="Q254" s="1"/>
       <c r="T254" t="s">
-        <v>1629</v>
+        <v>1626</v>
       </c>
       <c r="U254" t="s">
-        <v>1629</v>
+        <v>1626</v>
       </c>
     </row>
     <row r="255" spans="1:26">
@@ -19626,27 +19635,27 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="K266:L266"/>
-    <mergeCell ref="F267:G267"/>
-    <mergeCell ref="K270:L270"/>
-    <mergeCell ref="K273:L273"/>
-    <mergeCell ref="K276:L276"/>
-    <mergeCell ref="K279:L279"/>
-    <mergeCell ref="K282:L282"/>
-    <mergeCell ref="K285:L285"/>
-    <mergeCell ref="K288:L288"/>
-    <mergeCell ref="K291:L291"/>
-    <mergeCell ref="K294:L294"/>
-    <mergeCell ref="K297:L297"/>
-    <mergeCell ref="K300:L300"/>
-    <mergeCell ref="K303:L303"/>
-    <mergeCell ref="F304:H304"/>
     <mergeCell ref="L322:O322"/>
     <mergeCell ref="F305:H305"/>
     <mergeCell ref="K306:L306"/>
     <mergeCell ref="K309:L309"/>
     <mergeCell ref="K312:L312"/>
     <mergeCell ref="F320:I320"/>
+    <mergeCell ref="K294:L294"/>
+    <mergeCell ref="K297:L297"/>
+    <mergeCell ref="K300:L300"/>
+    <mergeCell ref="K303:L303"/>
+    <mergeCell ref="F304:H304"/>
+    <mergeCell ref="K279:L279"/>
+    <mergeCell ref="K282:L282"/>
+    <mergeCell ref="K285:L285"/>
+    <mergeCell ref="K288:L288"/>
+    <mergeCell ref="K291:L291"/>
+    <mergeCell ref="K266:L266"/>
+    <mergeCell ref="F267:G267"/>
+    <mergeCell ref="K270:L270"/>
+    <mergeCell ref="K273:L273"/>
+    <mergeCell ref="K276:L276"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Added relevancy condition exclusive breastfeeding note
</commit_message>
<xml_diff>
--- a/forms/app/infant_child.xlsx
+++ b/forms/app/infant_child.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2569" uniqueCount="1633">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2570" uniqueCount="1633">
   <si>
     <t>type</t>
   </si>
@@ -5333,9 +5333,6 @@
     <t>selected(${baby_times_breastfed_daily},"five_more_times_day")</t>
   </si>
   <si>
-    <t>not(selected(${baby_times_breastfed_daily},"five_more_times_day")) and (not(selected(${exclusive_breastfeeding},"yes")) or not(selected(${exclusive_breastfeeding_multiple_choice},"none")))</t>
-  </si>
-  <si>
     <t>exclusive_breastfeeding</t>
   </si>
   <si>
@@ -5361,6 +5358,9 @@
   </si>
   <si>
     <t xml:space="preserve">${age_days} &lt;= (${month} * 24) </t>
+  </si>
+  <si>
+    <t>not(selected(${baby_times_breastfed_daily},"five_more_times_day")) and ${age_days} &lt; (${month} * 6) and (not(selected(${exclusive_breastfeeding},"yes")) or not(selected(${exclusive_breastfeeding_multiple_choice},"none")))</t>
   </si>
 </sst>
 </file>
@@ -5480,9 +5480,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11035,7 +11035,7 @@
       <c r="D188" s="2" t="s">
         <v>479</v>
       </c>
-      <c r="F188" s="23" t="s">
+      <c r="F188" s="22" t="s">
         <v>401</v>
       </c>
     </row>
@@ -11163,8 +11163,8 @@
       <c r="E193" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="F193" s="24" t="s">
-        <v>1632</v>
+      <c r="F193" s="23" t="s">
+        <v>1631</v>
       </c>
       <c r="G193" s="1"/>
       <c r="H193" s="1"/>
@@ -11281,7 +11281,9 @@
       <c r="E197" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="F197" s="2"/>
+      <c r="F197" s="23" t="s">
+        <v>1631</v>
+      </c>
       <c r="G197" s="2"/>
       <c r="H197" s="2"/>
       <c r="I197" s="1"/>
@@ -11308,7 +11310,7 @@
         <v>1605</v>
       </c>
       <c r="F198" s="19" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
     </row>
     <row r="199" spans="1:17">
@@ -11325,7 +11327,7 @@
         <v>1603</v>
       </c>
       <c r="F199" s="19" t="s">
-        <v>1630</v>
+        <v>1629</v>
       </c>
     </row>
     <row r="200" spans="1:17">
@@ -11339,7 +11341,7 @@
       <c r="D200" s="18"/>
       <c r="F200" s="19"/>
       <c r="L200" t="s">
-        <v>1627</v>
+        <v>1626</v>
       </c>
     </row>
     <row r="201" spans="1:17">
@@ -11347,7 +11349,7 @@
         <v>167</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>1624</v>
+        <v>1623</v>
       </c>
       <c r="C201" s="2" t="s">
         <v>501</v>
@@ -11359,7 +11361,7 @@
         <v>171</v>
       </c>
       <c r="F201" s="2" t="s">
-        <v>1628</v>
+        <v>1627</v>
       </c>
       <c r="G201" s="2"/>
       <c r="H201" s="1"/>
@@ -11387,7 +11389,7 @@
         <v>1609</v>
       </c>
       <c r="F202" s="2" t="s">
-        <v>1629</v>
+        <v>1628</v>
       </c>
     </row>
     <row r="203" spans="1:17">
@@ -11478,7 +11480,7 @@
         <v>1619</v>
       </c>
       <c r="F206" s="2" t="s">
-        <v>1623</v>
+        <v>1632</v>
       </c>
     </row>
     <row r="207" spans="1:17">
@@ -12786,7 +12788,7 @@
         <v>139</v>
       </c>
       <c r="B254" s="1" t="s">
-        <v>1625</v>
+        <v>1624</v>
       </c>
       <c r="C254" s="10"/>
       <c r="D254" s="10"/>
@@ -12806,10 +12808,10 @@
       <c r="P254" s="1"/>
       <c r="Q254" s="1"/>
       <c r="T254" t="s">
-        <v>1626</v>
+        <v>1625</v>
       </c>
       <c r="U254" t="s">
-        <v>1626</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="255" spans="1:26">
@@ -13240,10 +13242,10 @@
       <c r="J266" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K266" s="22" t="s">
+      <c r="K266" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L266" s="22"/>
+      <c r="L266" s="24"/>
       <c r="M266" s="1"/>
       <c r="N266" s="1"/>
       <c r="O266" s="1"/>
@@ -13273,10 +13275,10 @@
         <v>684</v>
       </c>
       <c r="E267" s="1"/>
-      <c r="F267" s="22" t="s">
+      <c r="F267" s="24" t="s">
         <v>685</v>
       </c>
-      <c r="G267" s="22"/>
+      <c r="G267" s="24"/>
       <c r="H267" s="1"/>
       <c r="I267" s="1"/>
       <c r="J267" s="1"/>
@@ -13400,10 +13402,10 @@
       <c r="J270" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K270" s="22" t="s">
+      <c r="K270" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L270" s="22"/>
+      <c r="L270" s="24"/>
       <c r="M270" s="1"/>
       <c r="N270" s="1"/>
       <c r="O270" s="1"/>
@@ -13522,10 +13524,10 @@
       <c r="J273" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K273" s="22" t="s">
+      <c r="K273" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L273" s="22"/>
+      <c r="L273" s="24"/>
       <c r="M273" s="1"/>
       <c r="N273" s="1"/>
       <c r="O273" s="1"/>
@@ -13644,10 +13646,10 @@
       <c r="J276" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K276" s="22" t="s">
+      <c r="K276" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L276" s="22"/>
+      <c r="L276" s="24"/>
       <c r="M276" s="1"/>
       <c r="N276" s="1"/>
       <c r="O276" s="1"/>
@@ -13766,10 +13768,10 @@
       <c r="J279" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K279" s="22" t="s">
+      <c r="K279" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L279" s="22"/>
+      <c r="L279" s="24"/>
       <c r="M279" s="1"/>
       <c r="N279" s="1"/>
       <c r="O279" s="1"/>
@@ -13888,10 +13890,10 @@
       <c r="J282" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K282" s="22" t="s">
+      <c r="K282" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L282" s="22"/>
+      <c r="L282" s="24"/>
       <c r="M282" s="1"/>
       <c r="N282" s="1"/>
       <c r="O282" s="1"/>
@@ -14010,10 +14012,10 @@
       <c r="J285" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K285" s="22" t="s">
+      <c r="K285" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L285" s="22"/>
+      <c r="L285" s="24"/>
       <c r="M285" s="1"/>
       <c r="N285" s="1"/>
       <c r="O285" s="1"/>
@@ -14132,10 +14134,10 @@
       <c r="J288" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K288" s="22" t="s">
+      <c r="K288" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L288" s="22"/>
+      <c r="L288" s="24"/>
       <c r="M288" s="1"/>
       <c r="N288" s="1"/>
       <c r="O288" s="1"/>
@@ -14254,10 +14256,10 @@
       <c r="J291" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K291" s="22" t="s">
+      <c r="K291" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L291" s="22"/>
+      <c r="L291" s="24"/>
       <c r="M291" s="1"/>
       <c r="N291" s="1"/>
       <c r="O291" s="1"/>
@@ -14376,10 +14378,10 @@
       <c r="J294" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K294" s="22" t="s">
+      <c r="K294" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L294" s="22"/>
+      <c r="L294" s="24"/>
       <c r="M294" s="1"/>
       <c r="N294" s="1"/>
       <c r="O294" s="1"/>
@@ -14498,10 +14500,10 @@
       <c r="J297" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K297" s="22" t="s">
+      <c r="K297" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L297" s="22"/>
+      <c r="L297" s="24"/>
       <c r="M297" s="1"/>
       <c r="N297" s="1"/>
       <c r="O297" s="1"/>
@@ -14620,10 +14622,10 @@
       <c r="J300" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K300" s="22" t="s">
+      <c r="K300" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L300" s="22"/>
+      <c r="L300" s="24"/>
       <c r="M300" s="1"/>
       <c r="N300" s="1"/>
       <c r="O300" s="1"/>
@@ -14742,10 +14744,10 @@
       <c r="J303" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K303" s="22" t="s">
+      <c r="K303" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L303" s="22"/>
+      <c r="L303" s="24"/>
       <c r="M303" s="1"/>
       <c r="N303" s="1"/>
       <c r="O303" s="1"/>
@@ -14775,11 +14777,11 @@
         <v>669</v>
       </c>
       <c r="E304" s="1"/>
-      <c r="F304" s="22" t="s">
+      <c r="F304" s="24" t="s">
         <v>795</v>
       </c>
-      <c r="G304" s="22"/>
-      <c r="H304" s="22"/>
+      <c r="G304" s="24"/>
+      <c r="H304" s="24"/>
       <c r="I304" s="1"/>
       <c r="J304" s="1"/>
       <c r="K304" s="1"/>
@@ -14815,11 +14817,11 @@
       <c r="E305" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="F305" s="22" t="s">
+      <c r="F305" s="24" t="s">
         <v>795</v>
       </c>
-      <c r="G305" s="22"/>
-      <c r="H305" s="22"/>
+      <c r="G305" s="24"/>
+      <c r="H305" s="24"/>
       <c r="I305" s="1"/>
       <c r="J305" s="1"/>
       <c r="K305" s="1"/>
@@ -14864,10 +14866,10 @@
       <c r="J306" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K306" s="22" t="s">
+      <c r="K306" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L306" s="22"/>
+      <c r="L306" s="24"/>
       <c r="M306" s="1"/>
       <c r="N306" s="1"/>
       <c r="O306" s="1"/>
@@ -14986,10 +14988,10 @@
       <c r="J309" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K309" s="22" t="s">
+      <c r="K309" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L309" s="22"/>
+      <c r="L309" s="24"/>
       <c r="M309" s="1"/>
       <c r="N309" s="1"/>
       <c r="O309" s="1"/>
@@ -15108,10 +15110,10 @@
       <c r="J312" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="K312" s="22" t="s">
+      <c r="K312" s="24" t="s">
         <v>681</v>
       </c>
-      <c r="L312" s="22"/>
+      <c r="L312" s="24"/>
       <c r="M312" s="1"/>
       <c r="N312" s="1"/>
       <c r="O312" s="1"/>
@@ -15396,12 +15398,12 @@
         <v>845</v>
       </c>
       <c r="E320" s="1"/>
-      <c r="F320" s="22" t="s">
+      <c r="F320" s="24" t="s">
         <v>846</v>
       </c>
-      <c r="G320" s="22"/>
-      <c r="H320" s="22"/>
-      <c r="I320" s="22"/>
+      <c r="G320" s="24"/>
+      <c r="H320" s="24"/>
+      <c r="I320" s="24"/>
       <c r="J320" s="1"/>
       <c r="K320" s="1"/>
       <c r="L320" s="1"/>
@@ -15474,12 +15476,12 @@
       <c r="I322" s="1"/>
       <c r="J322" s="1"/>
       <c r="K322" s="1"/>
-      <c r="L322" s="22" t="s">
+      <c r="L322" s="24" t="s">
         <v>852</v>
       </c>
-      <c r="M322" s="22"/>
-      <c r="N322" s="22"/>
-      <c r="O322" s="22"/>
+      <c r="M322" s="24"/>
+      <c r="N322" s="24"/>
+      <c r="O322" s="24"/>
       <c r="P322" s="1"/>
       <c r="Q322" s="1"/>
       <c r="R322" s="6"/>
@@ -19635,27 +19637,27 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="K266:L266"/>
+    <mergeCell ref="F267:G267"/>
+    <mergeCell ref="K270:L270"/>
+    <mergeCell ref="K273:L273"/>
+    <mergeCell ref="K276:L276"/>
+    <mergeCell ref="K279:L279"/>
+    <mergeCell ref="K282:L282"/>
+    <mergeCell ref="K285:L285"/>
+    <mergeCell ref="K288:L288"/>
+    <mergeCell ref="K291:L291"/>
+    <mergeCell ref="K294:L294"/>
+    <mergeCell ref="K297:L297"/>
+    <mergeCell ref="K300:L300"/>
+    <mergeCell ref="K303:L303"/>
+    <mergeCell ref="F304:H304"/>
     <mergeCell ref="L322:O322"/>
     <mergeCell ref="F305:H305"/>
     <mergeCell ref="K306:L306"/>
     <mergeCell ref="K309:L309"/>
     <mergeCell ref="K312:L312"/>
     <mergeCell ref="F320:I320"/>
-    <mergeCell ref="K294:L294"/>
-    <mergeCell ref="K297:L297"/>
-    <mergeCell ref="K300:L300"/>
-    <mergeCell ref="K303:L303"/>
-    <mergeCell ref="F304:H304"/>
-    <mergeCell ref="K279:L279"/>
-    <mergeCell ref="K282:L282"/>
-    <mergeCell ref="K285:L285"/>
-    <mergeCell ref="K288:L288"/>
-    <mergeCell ref="K291:L291"/>
-    <mergeCell ref="K266:L266"/>
-    <mergeCell ref="F267:G267"/>
-    <mergeCell ref="K270:L270"/>
-    <mergeCell ref="K273:L273"/>
-    <mergeCell ref="K276:L276"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -20845,10 +20847,10 @@
       <c r="C84" s="1" t="s">
         <v>1561</v>
       </c>
-      <c r="D84" s="22" t="s">
+      <c r="D84" s="24" t="s">
         <v>1562</v>
       </c>
-      <c r="E84" s="22"/>
+      <c r="E84" s="24"/>
     </row>
     <row r="85" spans="1:6">
       <c r="A85" s="1" t="s">
@@ -20860,11 +20862,11 @@
       <c r="C85" s="1" t="s">
         <v>1563</v>
       </c>
-      <c r="D85" s="22" t="s">
+      <c r="D85" s="24" t="s">
         <v>1564</v>
       </c>
-      <c r="E85" s="22"/>
-      <c r="F85" s="22"/>
+      <c r="E85" s="24"/>
+      <c r="F85" s="24"/>
     </row>
     <row r="86" spans="1:6">
       <c r="A86" s="1" t="s">
@@ -20890,10 +20892,10 @@
       <c r="C87" s="1" t="s">
         <v>1567</v>
       </c>
-      <c r="D87" s="22" t="s">
+      <c r="D87" s="24" t="s">
         <v>1568</v>
       </c>
-      <c r="E87" s="22"/>
+      <c r="E87" s="24"/>
     </row>
     <row r="88" spans="1:6">
       <c r="A88" s="1" t="s">

</xml_diff>